<commit_message>
Daily tracker update 2026-10-13
</commit_message>
<xml_diff>
--- a/application_tracker.xlsx
+++ b/application_tracker.xlsx
@@ -471,7 +471,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>H1B Sponsor?</t>
+          <t>Green Card Sponsor</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -513,22 +513,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Senior Firmware Engineer</t>
+          <t>Senior Embedded Software Engineer</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Honeywell</t>
+          <t>Deere &amp; Company</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Remote, USA</t>
+          <t>Moline, IL</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes - proven</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
@@ -558,28 +558,28 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Senior Embedded Software Engineer</t>
+          <t>Embedded Software Engineer II</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Deere &amp; Company</t>
+          <t>Caterpillar</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Moline, IL</t>
+          <t>Peoria, IL</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes - proven</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>93.0</t>
+          <t>100.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -603,28 +603,28 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Embedded Software Engineer II</t>
+          <t>Controls Software Engineer</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Caterpillar</t>
+          <t>AGCO Corporation</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Peoria, IL</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Hesston, KS</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Yes - smaller</t>
         </is>
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>93.0</t>
+          <t>97.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -648,28 +648,28 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Firmware Engineer - Industrial Controls</t>
+          <t>Embedded Systems Engineer</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Rockwell Automation</t>
+          <t>Oshkosh Corporation</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Milwaukee, WI</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Oshkosh, WI</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>92.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -693,28 +693,28 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Embedded Systems Engineer</t>
+          <t>Software Engineer - Embedded Systems</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Oshkosh Corporation</t>
+          <t>Medtronic</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Oshkosh, WI</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Minneapolis, MN</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Yes - proven</t>
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>89.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -751,20 +751,20 @@
           <t>Cleveland, OH</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Yes - smaller</t>
         </is>
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>67.0</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -783,33 +783,33 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Software Engineer - Embedded Systems</t>
+          <t>Senior Firmware Engineer</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Medtronic</t>
+          <t>Honeywell</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Minneapolis, MN</t>
+          <t>Remote, USA</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes - proven</t>
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>67.0</t>
+          <t>86.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -828,33 +828,33 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Controls Software Engineer</t>
+          <t>Firmware Engineer - Industrial Controls</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AGCO Corporation</t>
+          <t>Rockwell Automation</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Hesston, KS</t>
+          <t>Milwaukee, WI</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes - proven</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>84.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -878,7 +878,11 @@
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Yes - proven</t>
+        </is>
+      </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
@@ -903,7 +907,11 @@
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Yes - proven</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
@@ -928,7 +936,11 @@
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Yes - proven</t>
+        </is>
+      </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
@@ -953,7 +965,11 @@
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Yes - proven</t>
+        </is>
+      </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
@@ -978,7 +994,11 @@
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Yes - proven</t>
+        </is>
+      </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
@@ -1003,7 +1023,11 @@
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Yes - proven</t>
+        </is>
+      </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
@@ -1028,7 +1052,11 @@
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Yes - proven</t>
+        </is>
+      </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
@@ -1053,7 +1081,11 @@
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
@@ -1078,7 +1110,11 @@
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Yes - proven</t>
+        </is>
+      </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
@@ -1103,7 +1139,11 @@
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Yes - proven</t>
+        </is>
+      </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
@@ -1128,7 +1168,11 @@
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Yes - smaller</t>
+        </is>
+      </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
@@ -1153,7 +1197,11 @@
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Yes - proven</t>
+        </is>
+      </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
@@ -1178,7 +1226,11 @@
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
@@ -1203,7 +1255,11 @@
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Yes - proven</t>
+        </is>
+      </c>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
@@ -1228,7 +1284,11 @@
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Yes - proven</t>
+        </is>
+      </c>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
@@ -1253,7 +1313,11 @@
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Yes - proven</t>
+        </is>
+      </c>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
@@ -1278,7 +1342,11 @@
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
@@ -1303,7 +1371,11 @@
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
@@ -1328,7 +1400,11 @@
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
@@ -1353,7 +1429,11 @@
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Yes - proven</t>
+        </is>
+      </c>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
@@ -1378,7 +1458,11 @@
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Yes - smaller</t>
+        </is>
+      </c>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr"/>
@@ -1403,7 +1487,11 @@
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Yes - smaller</t>
+        </is>
+      </c>
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
@@ -1428,7 +1516,11 @@
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Yes - smaller</t>
+        </is>
+      </c>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
@@ -1453,7 +1545,11 @@
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Yes - smaller</t>
+        </is>
+      </c>
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
@@ -1478,7 +1574,11 @@
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Yes - proven</t>
+        </is>
+      </c>
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
@@ -1503,7 +1603,11 @@
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Yes - proven</t>
+        </is>
+      </c>
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
@@ -1528,7 +1632,11 @@
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Yes - proven</t>
+        </is>
+      </c>
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr"/>
@@ -1553,7 +1661,11 @@
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Yes - proven</t>
+        </is>
+      </c>
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr"/>
@@ -1578,7 +1690,11 @@
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Yes - proven</t>
+        </is>
+      </c>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr"/>
@@ -1603,7 +1719,11 @@
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Yes - proven</t>
+        </is>
+      </c>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr"/>
@@ -1628,7 +1748,11 @@
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Yes - proven</t>
+        </is>
+      </c>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr"/>
@@ -1653,7 +1777,11 @@
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Yes - smaller</t>
+        </is>
+      </c>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
@@ -1678,7 +1806,11 @@
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr"/>
@@ -1703,7 +1835,11 @@
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Yes - smaller</t>
+        </is>
+      </c>
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
@@ -1728,7 +1864,11 @@
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Yes - proven</t>
+        </is>
+      </c>
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr"/>
@@ -1753,7 +1893,11 @@
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Yes - proven</t>
+        </is>
+      </c>
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr"/>
@@ -1778,7 +1922,11 @@
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Yes - proven</t>
+        </is>
+      </c>
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr"/>
@@ -1803,7 +1951,11 @@
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Yes - smaller</t>
+        </is>
+      </c>
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr"/>
@@ -1828,7 +1980,11 @@
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr"/>
@@ -1853,7 +2009,11 @@
         </is>
       </c>
       <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr"/>
@@ -1878,7 +2038,11 @@
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr"/>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Yes - smaller</t>
+        </is>
+      </c>
       <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr"/>
@@ -1903,7 +2067,11 @@
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
-      <c r="D51" t="inlineStr"/>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr"/>
@@ -1928,7 +2096,11 @@
         </is>
       </c>
       <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr"/>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Yes - smaller</t>
+        </is>
+      </c>
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr"/>
@@ -1953,7 +2125,11 @@
         </is>
       </c>
       <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr"/>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
       <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr"/>
@@ -1978,7 +2154,11 @@
         </is>
       </c>
       <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Yes - proven</t>
+        </is>
+      </c>
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
@@ -2003,7 +2183,11 @@
         </is>
       </c>
       <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr"/>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr"/>
@@ -2028,7 +2212,11 @@
         </is>
       </c>
       <c r="C56" t="inlineStr"/>
-      <c r="D56" t="inlineStr"/>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Yes - proven</t>
+        </is>
+      </c>
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr"/>
@@ -2053,7 +2241,11 @@
         </is>
       </c>
       <c r="C57" t="inlineStr"/>
-      <c r="D57" t="inlineStr"/>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Yes - proven</t>
+        </is>
+      </c>
       <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr"/>
@@ -2078,7 +2270,11 @@
         </is>
       </c>
       <c r="C58" t="inlineStr"/>
-      <c r="D58" t="inlineStr"/>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Yes - proven</t>
+        </is>
+      </c>
       <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr"/>
@@ -2103,7 +2299,11 @@
         </is>
       </c>
       <c r="C59" t="inlineStr"/>
-      <c r="D59" t="inlineStr"/>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
       <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr"/>
@@ -2128,7 +2328,11 @@
         </is>
       </c>
       <c r="C60" t="inlineStr"/>
-      <c r="D60" t="inlineStr"/>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr"/>

</xml_diff>